<commit_message>
feat(authentication): add VusuarioPermiso model and remove SphAutentication component
Add new view model for user permissions and clean up unused authentication component. The VusuarioPermiso model includes CRUD permissions for menu options and is now registered in SphericalContext.
</commit_message>
<xml_diff>
--- a/docs/Permisos/roles_permisos_menu.xlsx
+++ b/docs/Permisos/roles_permisos_menu.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documentos\Proyectos\Spherikal\Spherical\docs\Permisos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F32D3DAA-F1F5-4B10-AEBF-845D5FACF148}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40029B37-BBD4-49BA-A809-A9A5A0765158}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7DC664DC-C2CA-4666-9D32-D1A840F4E6E4}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="45">
   <si>
     <t>Rol</t>
   </si>
@@ -167,6 +167,9 @@
   </si>
   <si>
     <t>GALVAREZ</t>
+  </si>
+  <si>
+    <t>VistaPermisos</t>
   </si>
 </sst>
 </file>
@@ -570,20 +573,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC3366FB-FFBA-4F00-98F3-4AD8DB512A29}">
-  <dimension ref="B2:I25"/>
+  <dimension ref="B2:R25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.5546875" bestFit="1" customWidth="1"/>
     <col min="4" max="9" width="9.6640625" customWidth="1"/>
+    <col min="11" max="11" width="12.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="K2" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="s">
         <v>25</v>
       </c>
@@ -608,8 +615,32 @@
       <c r="I3" s="2" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="K3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="P3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="Q3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="R3" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
         <v>39</v>
       </c>
@@ -634,8 +665,32 @@
       <c r="I4" s="4" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="K4" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="M4" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="N4" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="O4" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="P4" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q4" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="R4" s="8" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B5" s="3" t="s">
         <v>41</v>
       </c>
@@ -658,12 +713,12 @@
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B8" s="2" t="s">
         <v>25</v>
       </c>
@@ -671,7 +726,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B9" s="5" t="s">
         <v>40</v>
       </c>
@@ -679,12 +734,12 @@
         <v>32</v>
       </c>
     </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B11" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B12" s="2" t="s">
         <v>26</v>
       </c>
@@ -710,7 +765,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B13" s="5" t="s">
         <v>40</v>
       </c>
@@ -736,12 +791,12 @@
         <v>37</v>
       </c>
     </row>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B15" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B16" s="2" t="s">
         <v>25</v>
       </c>
@@ -807,27 +862,27 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3FA8114-BD37-4EFA-BFB1-4258F065B7C2}">
-  <dimension ref="B2:Q37"/>
+  <dimension ref="B2:O37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="8" width="12.5546875" customWidth="1"/>
-    <col min="13" max="13" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="14.5546875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="5" customWidth="1"/>
-    <col min="19" max="19" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="5" customWidth="1"/>
+    <col min="17" max="17" width="16.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="M2" t="s">
+      <c r="K2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="s">
         <v>25</v>
       </c>
@@ -852,11 +907,11 @@
       <c r="I3" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="N3" t="s">
+      <c r="L3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
         <v>39</v>
       </c>
@@ -881,11 +936,11 @@
       <c r="I4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="O4" t="s">
+      <c r="M4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B5" s="3" t="s">
         <v>41</v>
       </c>
@@ -907,61 +962,61 @@
       <c r="I5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="O5" t="s">
+      <c r="M5" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="N6" t="s">
+    <row r="6" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="L6" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="O7" t="s">
+      <c r="M7" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B8" s="2" t="s">
         <v>25</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="N8" t="s">
+      <c r="L8" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B9" s="5" t="s">
         <v>40</v>
       </c>
       <c r="C9" t="s">
         <v>32</v>
       </c>
-      <c r="O9" t="s">
+      <c r="M9" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="O10" t="s">
+    <row r="10" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="M10" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="O11" t="s">
+    <row r="11" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="M11" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B12" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B13" s="1" t="s">
         <v>26</v>
       </c>
@@ -987,7 +1042,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B14" s="5" t="s">
         <v>40</v>
       </c>
@@ -1012,22 +1067,22 @@
       <c r="I14" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="P14" t="s">
+      <c r="N14" t="s">
         <v>11</v>
       </c>
-      <c r="Q14" t="s">
+      <c r="O14" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="P16" t="s">
+    <row r="16" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="N16" t="s">
         <v>11</v>
       </c>
-      <c r="Q16" t="s">
+      <c r="O16" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B17" s="1" t="s">
         <v>29</v>
       </c>
@@ -1037,31 +1092,31 @@
       <c r="D17" t="s">
         <v>8</v>
       </c>
+      <c r="K17" t="s">
+        <v>10</v>
+      </c>
+      <c r="L17" t="s">
+        <v>11</v>
+      </c>
       <c r="M17" t="s">
-        <v>10</v>
-      </c>
-      <c r="N17" t="s">
-        <v>11</v>
-      </c>
-      <c r="O17" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:15" x14ac:dyDescent="0.3">
       <c r="C18" t="s">
         <v>28</v>
       </c>
       <c r="D18" t="s">
         <v>30</v>
       </c>
-      <c r="P18" t="s">
+      <c r="N18" t="s">
         <v>11</v>
       </c>
-      <c r="Q18" t="s">
+      <c r="O18" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B20" s="1" t="s">
         <v>19</v>
       </c>
@@ -1071,14 +1126,14 @@
       <c r="D20" t="s">
         <v>26</v>
       </c>
-      <c r="P20" t="s">
+      <c r="N20" t="s">
         <v>11</v>
       </c>
-      <c r="Q20" t="s">
+      <c r="O20" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="21" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:15" x14ac:dyDescent="0.3">
       <c r="C21" t="s">
         <v>31</v>
       </c>
@@ -1086,7 +1141,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="23" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B23" s="1" t="s">
         <v>0</v>
       </c>
@@ -1097,7 +1152,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="24" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:15" x14ac:dyDescent="0.3">
       <c r="C24" t="s">
         <v>31</v>
       </c>
@@ -1105,7 +1160,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="26" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B26" s="1" t="s">
         <v>8</v>
       </c>
@@ -1119,7 +1174,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="27" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:15" x14ac:dyDescent="0.3">
       <c r="C27" t="s">
         <v>33</v>
       </c>
@@ -1127,7 +1182,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="28" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:15" x14ac:dyDescent="0.3">
       <c r="C28" t="s">
         <v>30</v>
       </c>
@@ -1141,7 +1196,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="29" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:15" x14ac:dyDescent="0.3">
       <c r="C29" t="s">
         <v>34</v>
       </c>

</xml_diff>

<commit_message>
feat(authentication): implement permission-based access control
- Add PermisoUsuarioDto for permission management
- Create PermisoService for permission checking
- Implement ApiServiceBase as base HTTP service
- Add authorization to ElementosController
- Update menu and element components to check permissions
- Add permission checks to UI actions
- Configure HttpClient services for new endpoints
</commit_message>
<xml_diff>
--- a/docs/Permisos/roles_permisos_menu.xlsx
+++ b/docs/Permisos/roles_permisos_menu.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documentos\Proyectos\Spherikal\Spherical\docs\Permisos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40029B37-BBD4-49BA-A809-A9A5A0765158}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5BF8D74-B1C3-4D0A-9B01-EC38F98F8A7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7DC664DC-C2CA-4666-9D32-D1A840F4E6E4}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="46">
   <si>
     <t>Rol</t>
   </si>
@@ -170,6 +170,9 @@
   </si>
   <si>
     <t>VistaPermisos</t>
+  </si>
+  <si>
+    <t>UsuarioRol</t>
   </si>
 </sst>
 </file>
@@ -835,7 +838,7 @@
     </row>
     <row r="23" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B23" s="1" t="s">
-        <v>10</v>
+        <v>45</v>
       </c>
     </row>
     <row r="24" spans="2:3" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
feat(inventory): add permission checks and improve UI for inventory management
- Implement permission checks for inventory movement and element management
- Restructure UI components to handle permission-based actions
- Add menu-based action controls for better user experience
- Move inventory movement page to new location
- Update permission service calls for both components
</commit_message>
<xml_diff>
--- a/docs/Permisos/roles_permisos_menu.xlsx
+++ b/docs/Permisos/roles_permisos_menu.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documentos\Proyectos\Spherikal\Spherical\docs\Permisos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5BF8D74-B1C3-4D0A-9B01-EC38F98F8A7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{943E5685-73F5-4488-8C99-E00FEF8A539A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7DC664DC-C2CA-4666-9D32-D1A840F4E6E4}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{7DC664DC-C2CA-4666-9D32-D1A840F4E6E4}"/>
   </bookViews>
   <sheets>
     <sheet name="Permisos Pantallas" sheetId="1" r:id="rId1"/>
-    <sheet name="Permisos Menu" sheetId="2" r:id="rId2"/>
+    <sheet name="Permisos Menu" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="33">
   <si>
     <t>Rol</t>
   </si>
@@ -55,45 +55,15 @@
     <t>x</t>
   </si>
   <si>
-    <t>Vista</t>
-  </si>
-  <si>
     <t>Anular</t>
   </si>
   <si>
     <t>Menu</t>
   </si>
   <si>
-    <t>Proyectos</t>
-  </si>
-  <si>
     <t>Usuario</t>
   </si>
   <si>
-    <t>&lt;&gt;</t>
-  </si>
-  <si>
-    <t>Permisos</t>
-  </si>
-  <si>
-    <t>Usuarios</t>
-  </si>
-  <si>
-    <t>Sistema</t>
-  </si>
-  <si>
-    <t>Roles</t>
-  </si>
-  <si>
-    <t>Tablas Basicas</t>
-  </si>
-  <si>
-    <t>Bodega</t>
-  </si>
-  <si>
-    <t>Opciones/Vista</t>
-  </si>
-  <si>
     <t>RolPermiso</t>
   </si>
   <si>
@@ -103,15 +73,6 @@
     <t>Descripcion</t>
   </si>
   <si>
-    <t>Tipo</t>
-  </si>
-  <si>
-    <t>P</t>
-  </si>
-  <si>
-    <t>M</t>
-  </si>
-  <si>
     <t>Id</t>
   </si>
   <si>
@@ -121,33 +82,12 @@
     <t>PermisoOpcion</t>
   </si>
   <si>
-    <t>P_UsuarioPlus</t>
-  </si>
-  <si>
     <t>PermisoMenu</t>
   </si>
   <si>
-    <t>M_Usuario</t>
-  </si>
-  <si>
-    <t>R_UsuarioPlus</t>
-  </si>
-  <si>
     <t>Sirve para</t>
   </si>
   <si>
-    <t>M_Sistema</t>
-  </si>
-  <si>
-    <t>M_Rol</t>
-  </si>
-  <si>
-    <t>V_Usuario</t>
-  </si>
-  <si>
-    <t>V_Rol</t>
-  </si>
-  <si>
     <t>o</t>
   </si>
   <si>
@@ -173,6 +113,27 @@
   </si>
   <si>
     <t>UsuarioRol</t>
+  </si>
+  <si>
+    <t>MInventarioElemento</t>
+  </si>
+  <si>
+    <t>MMvtoInterno</t>
+  </si>
+  <si>
+    <t>VistaMenu</t>
+  </si>
+  <si>
+    <t>PInventarioMenu</t>
+  </si>
+  <si>
+    <t>PMvtoInventarioMenu</t>
+  </si>
+  <si>
+    <t>Notas</t>
+  </si>
+  <si>
+    <t>Si se agrega el menu padre no se necesitan los hijos</t>
   </si>
 </sst>
 </file>
@@ -576,29 +537,32 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC3366FB-FFBA-4F00-98F3-4AD8DB512A29}">
-  <dimension ref="B2:R25"/>
+  <dimension ref="B2:R26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="1" max="1" width="2.109375" customWidth="1"/>
     <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="9" width="9.6640625" customWidth="1"/>
-    <col min="11" max="11" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="9" width="10.33203125" customWidth="1"/>
+    <col min="10" max="10" width="1.77734375" customWidth="1"/>
+    <col min="11" max="12" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="18" width="10.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>44</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="s">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>1</v>
@@ -613,16 +577,16 @@
         <v>4</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="K3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="L3" s="2" t="s">
         <v>10</v>
-      </c>
-      <c r="L3" s="2" t="s">
-        <v>20</v>
       </c>
       <c r="M3" s="2" t="s">
         <v>1</v>
@@ -637,18 +601,18 @@
         <v>4</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
-        <v>39</v>
+        <v>19</v>
       </c>
       <c r="C4" t="s">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>5</v>
@@ -666,13 +630,13 @@
         <v>5</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="K4" s="7" t="s">
-        <v>43</v>
+        <v>23</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>39</v>
+        <v>19</v>
       </c>
       <c r="M4" s="4" t="s">
         <v>5</v>
@@ -684,18 +648,18 @@
         <v>5</v>
       </c>
       <c r="P4" s="4" t="s">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="Q4" s="4" t="s">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="R4" s="8" t="s">
-        <v>37</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B5" s="3" t="s">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>5</v>
@@ -713,41 +677,65 @@
         <v>5</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>37</v>
+        <v>17</v>
+      </c>
+      <c r="K5" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="M5" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="N5" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="O5" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="P5" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q5" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="R5" s="8" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B8" s="2" t="s">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B9" s="5" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="C9" t="s">
-        <v>32</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B11" s="1" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B12" s="2" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>1</v>
@@ -762,18 +750,18 @@
         <v>4</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B13" s="5" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>39</v>
+        <v>19</v>
       </c>
       <c r="D13" s="4" t="s">
         <v>5</v>
@@ -785,76 +773,102 @@
         <v>5</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="15" spans="2:18" x14ac:dyDescent="0.3">
-      <c r="B15" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="2:18" x14ac:dyDescent="0.3">
+      <c r="B14" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I14" s="8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" spans="2:18" x14ac:dyDescent="0.3">
+      <c r="B16" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="2:18" x14ac:dyDescent="0.3">
-      <c r="B16" s="2" t="s">
+    <row r="17" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B17" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B18" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C18" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B20" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B21" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B22" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="24" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B24" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B17" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C17" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B19" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B20" s="2" t="s">
+    </row>
+    <row r="25" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B25" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C20" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="21" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B21" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C21" s="5" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="23" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B23" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="24" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B24" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B25" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="C25" s="6" t="s">
-        <v>42</v>
+    </row>
+    <row r="26" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B26" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -864,371 +878,218 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3FA8114-BD37-4EFA-BFB1-4258F065B7C2}">
-  <dimension ref="B2:O37"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99EBDE78-C6A1-413F-835E-D58DD452A461}">
+  <dimension ref="B2:H28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="8" width="12.5546875" customWidth="1"/>
-    <col min="11" max="11" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.5546875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="5" customWidth="1"/>
-    <col min="17" max="17" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="2.109375" customWidth="1"/>
+    <col min="2" max="2" width="19.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.33203125" customWidth="1"/>
+    <col min="5" max="5" width="1.77734375" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="7" max="7" width="14.5546875" customWidth="1"/>
+    <col min="8" max="8" width="18.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="K2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="2"/>
+      <c r="F3" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="3" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B3" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>3</v>
-      </c>
       <c r="G3" s="2" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I3" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="L3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="2:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="C4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" s="4"/>
+      <c r="F4" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B5" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="4"/>
+      <c r="F5" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="D6" s="4"/>
+    </row>
+    <row r="7" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B7" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B8" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B9" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B10" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="F10" t="s">
         <v>32</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="M4" t="s">
+    </row>
+    <row r="12" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B12" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B13" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="5" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B5" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="M5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="L6" t="s">
+      <c r="C13" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D13" s="2"/>
+    </row>
+    <row r="14" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B14" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D14" s="4"/>
+    </row>
+    <row r="15" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B15" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D15" s="4"/>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B17" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B18" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B19" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C19" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B7" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="M7" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B8" s="2" t="s">
+    <row r="21" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B21" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B22" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="23" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B23" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="24" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B24" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="26" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B26" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L8" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="9" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B9" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="C9" t="s">
-        <v>32</v>
-      </c>
-      <c r="M9" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="M10" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="11" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="M11" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="12" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B12" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="13" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B13" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="I13" s="2" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="14" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B14" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="H14" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="I14" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="N14" t="s">
-        <v>11</v>
-      </c>
-      <c r="O14" t="s">
+    </row>
+    <row r="27" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B27" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C27" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="N16" t="s">
-        <v>11</v>
-      </c>
-      <c r="O16" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="17" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B17" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C17" t="s">
-        <v>26</v>
-      </c>
-      <c r="D17" t="s">
-        <v>8</v>
-      </c>
-      <c r="K17" t="s">
-        <v>10</v>
-      </c>
-      <c r="L17" t="s">
-        <v>11</v>
-      </c>
-      <c r="M17" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="C18" t="s">
-        <v>28</v>
-      </c>
-      <c r="D18" t="s">
-        <v>30</v>
-      </c>
-      <c r="N18" t="s">
-        <v>11</v>
-      </c>
-      <c r="O18" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="20" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B20" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C20" t="s">
-        <v>0</v>
-      </c>
-      <c r="D20" t="s">
-        <v>26</v>
-      </c>
-      <c r="N20" t="s">
-        <v>11</v>
-      </c>
-      <c r="O20" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="21" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="C21" t="s">
-        <v>31</v>
-      </c>
-      <c r="D21" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="23" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B23" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C23" t="s">
-        <v>25</v>
-      </c>
-      <c r="D23" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="24" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="C24" t="s">
-        <v>31</v>
-      </c>
-      <c r="D24" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="26" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B26" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C26" t="s">
-        <v>25</v>
-      </c>
-      <c r="E26" t="s">
+    <row r="28" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B28" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C28" s="6" t="s">
         <v>22</v>
-      </c>
-      <c r="F26" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="27" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="C27" t="s">
-        <v>33</v>
-      </c>
-      <c r="E27" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="28" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="C28" t="s">
-        <v>30</v>
-      </c>
-      <c r="D28" t="s">
-        <v>33</v>
-      </c>
-      <c r="E28" t="s">
-        <v>24</v>
-      </c>
-      <c r="F28" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="29" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="C29" t="s">
-        <v>34</v>
-      </c>
-      <c r="D29" t="s">
-        <v>33</v>
-      </c>
-      <c r="E29" t="s">
-        <v>24</v>
-      </c>
-      <c r="F29" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="35" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B35" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C35" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="36" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="C36" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="37" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="C37" t="s">
-        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>